<commit_message>
fix: tighten pin assign workbench checks
</commit_message>
<xml_diff>
--- a/pin-assign-workbench/assets/pin-assign-template.xlsx
+++ b/pin-assign-workbench/assets/pin-assign-template.xlsx
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -108,6 +108,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -479,35 +482,35 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="36" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Pin Assign Workbench Template</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Keep source evidence, schematic order, and final net mapping separate. Fill Sources before final delivery.</t>
         </is>
       </c>
-      <c r="C1" s="1" t="n"/>
+      <c r="C1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1094,7 +1097,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1105,8 +1108,9 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1152,14 +1156,36 @@
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
+          <t>Intentional Duplicate Marker</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
           <t>Check Status</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n"/>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Y only when duplicate net is intentional and documented</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
@@ -1173,7 +1199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1184,6 +1210,7 @@
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1223,6 +1250,11 @@
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Source IDs</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>

</xml_diff>